<commit_message>
resaltando pronunciacion en vocalulary de freeCodeCamp
</commit_message>
<xml_diff>
--- a/developer_week_01.xlsx
+++ b/developer_week_01.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="238">
   <si>
     <t>approach</t>
   </si>
@@ -731,6 +731,9 @@
   </si>
   <si>
     <t>/raid/</t>
+  </si>
+  <si>
+    <t>/tok/</t>
   </si>
 </sst>
 </file>
@@ -1074,7 +1077,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2077,6 +2080,9 @@
       <c r="B17" t="s">
         <v>216</v>
       </c>
+      <c r="C17" t="s">
+        <v>237</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">

</xml_diff>